<commit_message>
QS: 82 Grammatikfehler korrigiert (mit die → mit den/der, in ohne Artikel, Dativ-Plural-Endungen)
</commit_message>
<xml_diff>
--- a/Kompetenzen und Maßnahmen/überfachliche Kompetenzen Vorklasse und Grundstufe Klassenstufe 0 bis 4 Version 5 QS.xlsx
+++ b/Kompetenzen und Maßnahmen/überfachliche Kompetenzen Vorklasse und Grundstufe Klassenstufe 0 bis 4 Version 5 QS.xlsx
@@ -541,17 +541,17 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in innere Körpersignale gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in den inneren Körpersignalen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in innere Körpersignale ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in den inneren Körpersignalen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in innere Körpersignale gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in den inneren Körpersignalen gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -584,17 +584,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in innere Körpersignale strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in den inneren Körpersignalen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in innere Körpersignale ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in den inneren Körpersignalen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in innere Körpersignale strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in den inneren Körpersignalen strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die inneren Körpersignale</t>
+          <t>kombiniert Atemübungen mit den inneren Körpersignalen</t>
         </is>
       </c>
     </row>
@@ -756,17 +756,17 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Gefühlsregungen im Bauch gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in den Gefühlsregungen im Bauch gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Gefühlsregungen im Bauch ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in den Gefühlsregungen im Bauch gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in Gefühlsregungen im Bauch gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in den Gefühlsregungen im Bauch gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -799,17 +799,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Gefühlsregungen im Bauch strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in den Gefühlsregungen im Bauch strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Gefühlsregungen im Bauch ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in den Gefühlsregungen im Bauch strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in Gefühlsregungen im Bauch strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in den Gefühlsregungen im Bauch strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Gefühlsregungen im Bauch</t>
+          <t>kombiniert Atemübungen mit den Gefühlsregungen im Bauch</t>
         </is>
       </c>
     </row>
@@ -971,17 +971,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Muskelspannung in Schultern und Nacken gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in der Muskelspannung in Schultern und Nacken gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Muskelspannung in Schultern und Nacken ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in der Muskelspannung in Schultern und Nacken gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in Muskelspannung in Schultern und Nacken gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in der Muskelspannung in Schultern und Nacken gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Muskelspannung in Schultern und Nacken strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in der Muskelspannung in Schultern und Nacken strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Muskelspannung in Schultern und Nacken ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in der Muskelspannung in Schultern und Nacken strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in Muskelspannung in Schultern und Nacken strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in der Muskelspannung in Schultern und Nacken strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Muskelspannung in Schultern und Nacken</t>
+          <t>kombiniert Atemübungen mit der Muskelspannung in Schultern und Nacken</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Atmung in Ruhe und Bewegung gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in der Atmung in Ruhe und Bewegung gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Atmung in Ruhe und Bewegung ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in der Atmung in Ruhe und Bewegung gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in Atmung in Ruhe und Bewegung gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in der Atmung in Ruhe und Bewegung gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1229,17 +1229,17 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Atmung in Ruhe und Bewegung strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in der Atmung in Ruhe und Bewegung strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Atmung in Ruhe und Bewegung ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in der Atmung in Ruhe und Bewegung strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in Atmung in Ruhe und Bewegung strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in der Atmung in Ruhe und Bewegung strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Atmung in Ruhe und Bewegung</t>
+          <t>kombiniert Atemübungen mit der Atmung in Ruhe und Bewegung</t>
         </is>
       </c>
     </row>
@@ -1401,17 +1401,17 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Sinneseindrücke der Haut gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in den Sinneseindrücken der Haut gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Sinneseindrücke der Haut ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in den Sinneseindrücken der Haut gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in Sinneseindrücke der Haut gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in den Sinneseindrücken der Haut gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Sinneseindrücke der Haut strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in den Sinneseindrücken der Haut strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Sinneseindrücke der Haut ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in den Sinneseindrücken der Haut strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in Sinneseindrücke der Haut strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in den Sinneseindrücken der Haut strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Sinneseindrücke der Haut</t>
+          <t>kombiniert Atemübungen mit den Sinneseindrücken der Haut</t>
         </is>
       </c>
     </row>
@@ -1616,17 +1616,17 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Körperhaltung beim Sitzen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in der Körperhaltung beim Sitzen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Körperhaltung beim Sitzen ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in der Körperhaltung beim Sitzen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in Körperhaltung beim Sitzen gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in der Körperhaltung beim Sitzen gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1659,17 +1659,17 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Körperhaltung beim Sitzen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in der Körperhaltung beim Sitzen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Körperhaltung beim Sitzen ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in der Körperhaltung beim Sitzen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in Körperhaltung beim Sitzen strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in der Körperhaltung beim Sitzen strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Körperhaltung beim Sitzen</t>
+          <t>kombiniert Atemübungen mit der Körperhaltung beim Sitzen</t>
         </is>
       </c>
     </row>
@@ -1831,17 +1831,17 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Bewegungsimpulse in den Händen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
+          <t>wiederkehrende Veränderungen in den Bewegungsimpulsen in den Händen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>wiederkehrende Veränderungen in Bewegungsimpulse in den Händen ##gezielt## beschreiben und einfache ##Handlungsimpulse## ableiten</t>
+          <t>wiederkehrende Veränderungen in den Bewegungsimpulsen in den Händen gezielt beschreiben und einfache Handlungsimpulse ableiten</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>beschreibt wiederkehrende Veränderungen in Bewegungsimpulse in den Händen gezielt und leitet einfache Handlungsimpulse ab</t>
+          <t>beschreibt wiederkehrende Veränderungen in den Bewegungsimpulsen in den Händen gezielt und leitet einfache Handlungsimpulse ab</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1874,17 +1874,17 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Bewegungsimpulse in den Händen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
+          <t>Veränderungen in den Bewegungsimpulsen in den Händen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Veränderungen in Bewegungsimpulse in den Händen ##strukturiert## beobachten und passende ##Selbstregulationsideen## auswählen</t>
+          <t>Veränderungen in den Bewegungsimpulsen in den Händen strukturiert beobachten und passende Selbstregulationsideen auswählen</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>beobachtet Veränderungen in Bewegungsimpulse in den Händen strukturiert und wählt passende Selbstregulationsideen aus</t>
+          <t>beobachtet Veränderungen in den Bewegungsimpulsen in den Händen strukturiert und wählt passende Selbstregulationsideen aus</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Bewegungsimpulse in den Händen</t>
+          <t>kombiniert Atemübungen mit den Bewegungsimpulsen in den Händen</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Ruhe- und Aktivitätsphasen</t>
+          <t>kombiniert Atemübungen mit den Ruhe- und Aktivitätsphasen</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>kombiniert Atemübungen mit die Bedürfnissignale wie Hunger oder Durst</t>
+          <t>kombiniert Atemübungen mit den Bedürfnissignale wie Hunger oder Durst</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Aufmerksamkeit bei Lautstärke</t>
+          <t>verknüpft Selbstinstruktionen mit der Aufmerksamkeit bei Lautstärke</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Aufmerksamkeit bei Lautstärke</t>
+          <t>plant Ersatzhandlungen im Umgang mit der Aufmerksamkeit bei Lautstärke</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5124,7 @@
       </c>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Impulskontrolle im Spiel</t>
+          <t>verknüpft Selbstinstruktionen mit der Impulskontrolle im Spiel</t>
         </is>
       </c>
     </row>
@@ -5167,7 +5167,7 @@
       </c>
       <c r="I110" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Impulskontrolle im Spiel</t>
+          <t>plant Ersatzhandlungen im Umgang mit der Impulskontrolle im Spiel</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="I114" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Übergänge zwischen Aktivitäten</t>
+          <t>verknüpft Selbstinstruktionen mit den Übergänge zwischen Aktivitäten</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="I115" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Übergänge zwischen Aktivitäten</t>
+          <t>plant Ersatzhandlungen im Umgang mit den Übergänge zwischen Aktivitäten</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="I119" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Arbeitsbeginnsrituale</t>
+          <t>verknüpft Selbstinstruktionen mit den Arbeitsbeginnsrituale</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="I120" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Arbeitsbeginnsrituale</t>
+          <t>plant Ersatzhandlungen im Umgang mit den Arbeitsbeginnsrituale</t>
         </is>
       </c>
     </row>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Pausengestaltung</t>
+          <t>verknüpft Selbstinstruktionen mit der Pausengestaltung</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I125" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Pausengestaltung</t>
+          <t>plant Ersatzhandlungen im Umgang mit der Pausengestaltung</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die emotionalen Reaktionen</t>
+          <t>verknüpft Selbstinstruktionen mit den emotionalen Reaktionen</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6242,7 @@
       </c>
       <c r="I135" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die emotionalen Reaktionen</t>
+          <t>plant Ersatzhandlungen im Umgang mit den emotionalen Reaktionen</t>
         </is>
       </c>
     </row>
@@ -6629,7 +6629,7 @@
       </c>
       <c r="I144" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Selbstgespräche zur Beruhigung</t>
+          <t>verknüpft Selbstinstruktionen mit den Selbstgespräche zur Beruhigung</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="I145" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Selbstgespräche zur Beruhigung</t>
+          <t>plant Ersatzhandlungen im Umgang mit den Selbstgespräche zur Beruhigung</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6844,7 @@
       </c>
       <c r="I149" s="3" t="inlineStr">
         <is>
-          <t>verknüpft Selbstinstruktionen mit die Entspannungsstrategien</t>
+          <t>verknüpft Selbstinstruktionen mit den Entspannungsstrategien</t>
         </is>
       </c>
     </row>
@@ -6887,7 +6887,7 @@
       </c>
       <c r="I150" s="3" t="inlineStr">
         <is>
-          <t>plant Ersatzhandlungen im Umgang mit die Entspannungsstrategien</t>
+          <t>plant Ersatzhandlungen im Umgang mit den Entspannungsstrategien</t>
         </is>
       </c>
     </row>

</xml_diff>